<commit_message>
Documentation: descriptions for the intake and employer tables
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Documentation/cercit-database-schema.xlsx
+++ b/Documentation/cercit-database-schema.xlsx
@@ -580,7 +580,11 @@
           <t>customers</t>
         </is>
       </c>
-      <c r="C2" s="2" t="inlineStr"/>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>One row per borrower: identity, contact and work details for a person applying for a car loan. PAN and mobile are stored encrypted; the plain columns are emptied by a trigger on every write.</t>
+        </is>
+      </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
           <t>001_schema.sql</t>
@@ -610,7 +614,11 @@
           <t>customer_addresses</t>
         </is>
       </c>
-      <c r="C3" s="2" t="inlineStr"/>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>One address of a customer, at most one row per type (permanent, current, office). Written by the customer journey's address step; saving again overwrites the row and clears its verified flag.</t>
+        </is>
+      </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
           <t>043_customer_onboarding.sql</t>
@@ -640,7 +648,11 @@
           <t>customer_consents</t>
         </is>
       </c>
-      <c r="C4" s="2" t="inlineStr"/>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>One row each time a customer accepts a consent wording, such as processing the application or pulling the credit report. It keeps a fingerprint of the exact text accepted; each acceptance adds a new row.</t>
+        </is>
+      </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
           <t>043_customer_onboarding.sql</t>
@@ -670,7 +682,11 @@
           <t>consent_texts</t>
         </is>
       </c>
-      <c r="C5" s="2" t="inlineStr"/>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>Reference table of consent wordings, one row per purpose and version. Seeded with the application-processing and credit-bureau consents; the current version is what customers see and accept.</t>
+        </is>
+      </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
           <t>043_customer_onboarding.sql</t>
@@ -702,7 +718,11 @@
           <t>applications</t>
         </is>
       </c>
-      <c r="C6" s="2" t="inlineStr"/>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>The central table: one row per car loan application, from draft to decision and disbursal. It holds the loan ask, declared income and expenses, stage dates, and the employer category used for pricing.</t>
+        </is>
+      </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
           <t>001_schema.sql</t>
@@ -732,7 +752,11 @@
           <t>application_detail_groups</t>
         </is>
       </c>
-      <c r="C7" s="2" t="inlineStr"/>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>One row per application per group of details (personal, address, work). It keeps what the system pre-filled from the documents, what the customer confirmed, and which fields they changed; confirming again overwrites the row.</t>
+        </is>
+      </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
           <t>046_customer_details_submit.sql</t>
@@ -764,7 +788,11 @@
           <t>application_stage_events</t>
         </is>
       </c>
-      <c r="C8" s="2" t="inlineStr"/>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>Timeline of stages an application has reached, one row per stage event, read by the customer's tracking page. Rows are only added, and a RECEIVED row starts the automatic document review.</t>
+        </is>
+      </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
           <t>046_customer_details_submit.sql</t>
@@ -796,7 +824,11 @@
           <t>application_document_requirements</t>
         </is>
       </c>
-      <c r="C9" s="2" t="inlineStr"/>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>Document checklist for a customer-journey application: one row per document type, with whether it is needed and where it stands. Created from document_types when the application starts; its first row marks the application's origin as CUSTOMER.</t>
+        </is>
+      </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
           <t>043_customer_onboarding.sql</t>
@@ -830,7 +862,11 @@
           <t>vehicles</t>
         </is>
       </c>
-      <c r="C10" s="2" t="inlineStr"/>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>The car being financed on an application, with its price breakdown and dealer. Part of the original schema; the application points back to it through vehicle_id.</t>
+        </is>
+      </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
           <t>001_schema.sql</t>
@@ -860,7 +896,11 @@
           <t>vehicle_quotations</t>
         </is>
       </c>
-      <c r="C11" s="2" t="inlineStr"/>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>The car details from the customer journey, one row per application: copied from the dealer's quotation or typed in by the customer. Saving again overwrites the row and updates the loan amount and tenure on the application.</t>
+        </is>
+      </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
           <t>043_customer_onboarding.sql</t>
@@ -890,7 +930,11 @@
           <t>dealers</t>
         </is>
       </c>
-      <c r="C12" s="2" t="inlineStr"/>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>Master list of car dealers, one row per dealership, seeded by car make and city. Used to link vehicles and quotations to a known dealer.</t>
+        </is>
+      </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
           <t>001_schema.sql</t>
@@ -920,7 +964,11 @@
           <t>states</t>
         </is>
       </c>
-      <c r="C13" s="2" t="inlineStr"/>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>Reference list of Indian states and union territories, one row each. It marks where the lender operates and holds each state's road tax rate.</t>
+        </is>
+      </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
           <t>001_schema.sql</t>
@@ -1794,7 +1842,11 @@
           <t>employers</t>
         </is>
       </c>
-      <c r="C38" s="2" t="inlineStr"/>
+      <c r="C38" s="2" t="inlineStr">
+        <is>
+          <t>Employer Master: one row per employer, with its identifiers, check results and A/B/C category, which drives the rate loading, LTV and tenure caps and processing fee. Closed to the API; read and changed only through functions.</t>
+        </is>
+      </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
           <t>069_employer_master.sql</t>
@@ -1824,7 +1876,11 @@
           <t>employer_checks</t>
         </is>
       </c>
-      <c r="C39" s="2" t="inlineStr"/>
+      <c r="C39" s="2" t="inlineStr">
+        <is>
+          <t>Log of every check run on an employer, one row per check per run, with its result and source. Rows are only added; the latest row per check decides whether the employer counts as verified.</t>
+        </is>
+      </c>
       <c r="D39" s="2" t="inlineStr">
         <is>
           <t>069_employer_master.sql</t>
@@ -1856,7 +1912,11 @@
           <t>employer_category_changes</t>
         </is>
       </c>
-      <c r="C40" s="2" t="inlineStr"/>
+      <c r="C40" s="2" t="inlineStr">
+        <is>
+          <t>Requests to change an employer's A/B/C category, one row per request. One person asks and a different person approves or rejects; only one open request per employer at a time.</t>
+        </is>
+      </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
           <t>069_employer_master.sql</t>
@@ -1888,7 +1948,11 @@
           <t>employer_reference_list</t>
         </is>
       </c>
-      <c r="C41" s="2" t="inlineStr"/>
+      <c r="C41" s="2" t="inlineStr">
+        <is>
+          <t>Maintained lists the employer checks compare with: government and PSU bodies, and NSE/BSE listed companies. One row per list per employer name.</t>
+        </is>
+      </c>
       <c r="D41" s="2" t="inlineStr">
         <is>
           <t>069_employer_master.sql</t>
@@ -1920,7 +1984,11 @@
           <t>employer_master_settings</t>
         </is>
       </c>
-      <c r="C42" s="2" t="inlineStr"/>
+      <c r="C42" s="2" t="inlineStr">
+        <is>
+          <t>Single-row settings table saying which provider runs the employer company checks. SIMULATED today; a live MCA provider is meant to replace it later.</t>
+        </is>
+      </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
           <t>069_employer_master.sql</t>
@@ -1952,7 +2020,11 @@
           <t>employer_category_pricing</t>
         </is>
       </c>
-      <c r="C43" s="2" t="inlineStr"/>
+      <c r="C43" s="2" t="inlineStr">
+        <is>
+          <t>Pricing terms per employer category (A, B, C) and policy version: rate loading, LTV and tenure caps, and processing fee. The engine adds these on top of the bureau band; readable by anyone.</t>
+        </is>
+      </c>
       <c r="D43" s="2" t="inlineStr">
         <is>
           <t>011_employer_category_pricing.sql</t>
@@ -4235,7 +4307,7 @@
       <c r="J2" s="2" t="inlineStr"/>
       <c r="K2" s="2" t="inlineStr">
         <is>
-          <t>Internal primary key</t>
+          <t>Internal key.</t>
         </is>
       </c>
     </row>
@@ -4274,7 +4346,7 @@
       <c r="J3" s="2" t="inlineStr"/>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>Full name as per PAN card</t>
+          <t>Customer's full name as one text.</t>
         </is>
       </c>
     </row>
@@ -4317,7 +4389,7 @@
       <c r="J4" s="2" t="inlineStr"/>
       <c r="K4" s="2" t="inlineStr">
         <is>
-          <t>Primary identity; OTP verified</t>
+          <t>Customer's email address; unique across customers.</t>
         </is>
       </c>
     </row>
@@ -4356,7 +4428,7 @@
       <c r="J5" s="2" t="inlineStr"/>
       <c r="K5" s="2" t="inlineStr">
         <is>
-          <t>Contact number (not verified in Phase 1)</t>
+          <t>Write-only inbox. A trigger encrypts it into mobile_enc and empties this; a CHECK keeps it empty. Read mobile_last4 or fn_customer_pii.</t>
         </is>
       </c>
     </row>
@@ -4395,7 +4467,7 @@
       <c r="J6" s="2" t="inlineStr"/>
       <c r="K6" s="2" t="inlineStr">
         <is>
-          <t>PAN extracted from uploaded PAN card</t>
+          <t>Write-only inbox. A trigger encrypts it into pan_enc and empties this; a CHECK keeps it empty. Read pan_last4 or fn_customer_pii.</t>
         </is>
       </c>
     </row>
@@ -4434,7 +4506,7 @@
       <c r="J7" s="2" t="inlineStr"/>
       <c r="K7" s="2" t="inlineStr">
         <is>
-          <t>Last 4 digits of Aadhaar (full number never stored)</t>
+          <t>Last four digits of the Aadhaar number only; the full number is not stored.</t>
         </is>
       </c>
     </row>
@@ -4473,7 +4545,7 @@
       <c r="J8" s="2" t="inlineStr"/>
       <c r="K8" s="2" t="inlineStr">
         <is>
-          <t>DOB from KYC documents</t>
+          <t>Customer's date of birth.</t>
         </is>
       </c>
     </row>
@@ -4512,7 +4584,7 @@
       <c r="J9" s="2" t="inlineStr"/>
       <c r="K9" s="2" t="inlineStr">
         <is>
-          <t>Age calculated at application date (min 21)</t>
+          <t>Customer's age in years at the time of applying.</t>
         </is>
       </c>
     </row>
@@ -4551,7 +4623,7 @@
       <c r="J10" s="2" t="inlineStr"/>
       <c r="K10" s="2" t="inlineStr">
         <is>
-          <t>M / F / OTHER — from KYC</t>
+          <t>Gender; the details step accepts MALE | FEMALE | OTHER.</t>
         </is>
       </c>
     </row>
@@ -4590,7 +4662,7 @@
       <c r="J11" s="2" t="inlineStr"/>
       <c r="K11" s="2" t="inlineStr">
         <is>
-          <t>Current address from Aadhaar</t>
+          <t>First address line on the original customer record; full addresses by type are kept in customer_addresses.</t>
         </is>
       </c>
     </row>
@@ -4629,7 +4701,7 @@
       <c r="J12" s="2" t="inlineStr"/>
       <c r="K12" s="2" t="inlineStr">
         <is>
-          <t>Address line 2</t>
+          <t>Second address line on the original customer record.</t>
         </is>
       </c>
     </row>
@@ -4668,7 +4740,7 @@
       <c r="J13" s="2" t="inlineStr"/>
       <c r="K13" s="2" t="inlineStr">
         <is>
-          <t>City name</t>
+          <t>City of the address on the customer record.</t>
         </is>
       </c>
     </row>
@@ -4715,7 +4787,7 @@
       <c r="J14" s="2" t="inlineStr"/>
       <c r="K14" s="2" t="inlineStr">
         <is>
-          <t>State code</t>
+          <t>State code of the customer's address; links to states.</t>
         </is>
       </c>
     </row>
@@ -4754,7 +4826,7 @@
       <c r="J15" s="2" t="inlineStr"/>
       <c r="K15" s="2" t="inlineStr">
         <is>
-          <t>6-digit pincode</t>
+          <t>6-digit PIN code of the address on the customer record.</t>
         </is>
       </c>
     </row>
@@ -4793,7 +4865,7 @@
       <c r="J16" s="2" t="inlineStr"/>
       <c r="K16" s="2" t="inlineStr">
         <is>
-          <t>Employer as per salary slip / Form 16</t>
+          <t>Employer name as the customer gave it; used to find the employer in the Employer Master.</t>
         </is>
       </c>
     </row>
@@ -4832,7 +4904,7 @@
       <c r="J17" s="2" t="inlineStr"/>
       <c r="K17" s="2" t="inlineStr">
         <is>
-          <t>SALARIED (Phase 1 only)</t>
+          <t>Type of employment, e.g. SALARIED. Phase 1 covers salaried applicants only.</t>
         </is>
       </c>
     </row>
@@ -4875,7 +4947,7 @@
       <c r="J18" s="2" t="inlineStr"/>
       <c r="K18" s="2" t="inlineStr">
         <is>
-          <t>True after OTP verification</t>
+          <t>True once the customer proved the email with the emailed code.</t>
         </is>
       </c>
     </row>
@@ -4914,7 +4986,7 @@
       <c r="J19" s="2" t="inlineStr"/>
       <c r="K19" s="2" t="inlineStr">
         <is>
-          <t>Supabase Auth user ID for login/OTP</t>
+          <t>Login account linked to this customer.</t>
         </is>
       </c>
     </row>
@@ -4957,7 +5029,7 @@
       <c r="J20" s="2" t="inlineStr"/>
       <c r="K20" s="2" t="inlineStr">
         <is>
-          <t>Record creation timestamp</t>
+          <t>When the row was created.</t>
         </is>
       </c>
     </row>
@@ -5000,7 +5072,7 @@
       <c r="J21" s="2" t="inlineStr"/>
       <c r="K21" s="2" t="inlineStr">
         <is>
-          <t>Last update timestamp</t>
+          <t>When the row was last changed; set automatically.</t>
         </is>
       </c>
     </row>
@@ -5039,7 +5111,7 @@
       <c r="J22" s="2" t="inlineStr"/>
       <c r="K22" s="2" t="inlineStr">
         <is>
-          <t>Pan enc</t>
+          <t>PAN encrypted with the PII key. Read only through fn_customer_pii, which checks the staff role and logs each reveal.</t>
         </is>
       </c>
     </row>
@@ -5078,7 +5150,7 @@
       <c r="J23" s="2" t="inlineStr"/>
       <c r="K23" s="2" t="inlineStr">
         <is>
-          <t>Pan hash</t>
+          <t>Keyed hash (HMAC-SHA256) of the PAN; lets the system find a customer by PAN and keeps PAN unique.</t>
         </is>
       </c>
     </row>
@@ -5117,7 +5189,7 @@
       <c r="J24" s="2" t="inlineStr"/>
       <c r="K24" s="2" t="inlineStr">
         <is>
-          <t>Pan last4</t>
+          <t>Last four characters of the PAN, kept plain for masked display (XXXXXX234F).</t>
         </is>
       </c>
     </row>
@@ -5156,7 +5228,7 @@
       <c r="J25" s="2" t="inlineStr"/>
       <c r="K25" s="2" t="inlineStr">
         <is>
-          <t>Mobile enc</t>
+          <t>Mobile number encrypted with the PII key; a CHECK requires it on every row. Read only through fn_customer_pii.</t>
         </is>
       </c>
     </row>
@@ -5195,7 +5267,7 @@
       <c r="J26" s="2" t="inlineStr"/>
       <c r="K26" s="2" t="inlineStr">
         <is>
-          <t>Mobile last4</t>
+          <t>Last four digits of the mobile, kept plain for masked display.</t>
         </is>
       </c>
     </row>
@@ -5234,7 +5306,7 @@
       <c r="J27" s="2" t="inlineStr"/>
       <c r="K27" s="2" t="inlineStr">
         <is>
-          <t>Designation</t>
+          <t>Customer's job title at the current employer.</t>
         </is>
       </c>
     </row>
@@ -5273,7 +5345,7 @@
       <c r="J28" s="2" t="inlineStr"/>
       <c r="K28" s="2" t="inlineStr">
         <is>
-          <t>Years in current job</t>
+          <t>Years in the current job, 0 to 60; cannot be more than total work experience.</t>
         </is>
       </c>
     </row>
@@ -5312,7 +5384,7 @@
       <c r="J29" s="2" t="inlineStr"/>
       <c r="K29" s="2" t="inlineStr">
         <is>
-          <t>Total work experience years</t>
+          <t>Total years of work experience, 0 to 60.</t>
         </is>
       </c>
     </row>
@@ -5351,7 +5423,7 @@
       <c r="J30" s="2" t="inlineStr"/>
       <c r="K30" s="2" t="inlineStr">
         <is>
-          <t>Salary bank name</t>
+          <t>Bank where the customer's salary is credited.</t>
         </is>
       </c>
     </row>
@@ -5390,7 +5462,7 @@
       <c r="J31" s="2" t="inlineStr"/>
       <c r="K31" s="2" t="inlineStr">
         <is>
-          <t>Residence type</t>
+          <t>Type of home: OWNED | RENTED | PARENTAL | COMPANY_PROVIDED, or empty.</t>
         </is>
       </c>
     </row>
@@ -5429,7 +5501,7 @@
       <c r="J32" s="2" t="inlineStr"/>
       <c r="K32" s="2" t="inlineStr">
         <is>
-          <t>First name</t>
+          <t>Customer's first name, captured at the start of the customer journey.</t>
         </is>
       </c>
     </row>
@@ -5468,7 +5540,7 @@
       <c r="J33" s="2" t="inlineStr"/>
       <c r="K33" s="2" t="inlineStr">
         <is>
-          <t>Middle name</t>
+          <t>Customer's middle name or initial, if any.</t>
         </is>
       </c>
     </row>
@@ -5507,7 +5579,7 @@
       <c r="J34" s="2" t="inlineStr"/>
       <c r="K34" s="2" t="inlineStr">
         <is>
-          <t>Last name</t>
+          <t>Customer's last name or initial.</t>
         </is>
       </c>
     </row>
@@ -5546,7 +5618,7 @@
       <c r="J35" s="2" t="inlineStr"/>
       <c r="K35" s="2" t="inlineStr">
         <is>
-          <t>When mobile verified</t>
+          <t>When the mobile number check (OTP) passed.</t>
         </is>
       </c>
     </row>
@@ -5585,7 +5657,7 @@
       <c r="J36" s="2" t="inlineStr"/>
       <c r="K36" s="2" t="inlineStr">
         <is>
-          <t>Mobile verification method</t>
+          <t>How the mobile was checked: SMS | SIMULATED. OTP is simulated until an SMS provider is connected.</t>
         </is>
       </c>
     </row>
@@ -5624,7 +5696,7 @@
       <c r="J37" s="2" t="inlineStr"/>
       <c r="K37" s="2" t="inlineStr">
         <is>
-          <t>Father name</t>
+          <t>Father's name, given in the personal details step.</t>
         </is>
       </c>
     </row>
@@ -5663,7 +5735,7 @@
       <c r="J38" s="2" t="inlineStr"/>
       <c r="K38" s="2" t="inlineStr">
         <is>
-          <t>Marital status</t>
+          <t>Marital status; the details step accepts SINGLE | MARRIED | OTHER.</t>
         </is>
       </c>
     </row>
@@ -5702,7 +5774,7 @@
       <c r="J39" s="2" t="inlineStr"/>
       <c r="K39" s="2" t="inlineStr">
         <is>
-          <t>Date of joining</t>
+          <t>Date the customer joined the current employer.</t>
         </is>
       </c>
     </row>
@@ -5741,7 +5813,7 @@
       <c r="J40" s="2" t="inlineStr"/>
       <c r="K40" s="2" t="inlineStr">
         <is>
-          <t>Employer category</t>
+          <t>Employer type the customer picked: PRIVATE_LTD | PUBLIC_LTD | MNC | GOVERNMENT | PSU | PARTNERSHIP | PROPRIETORSHIP | OTHER. Not the A/B/C category.</t>
         </is>
       </c>
     </row>
@@ -5780,7 +5852,7 @@
       <c r="J41" s="2" t="inlineStr"/>
       <c r="K41" s="2" t="inlineStr">
         <is>
-          <t>Mobile hash</t>
+          <t>Keyed hash of the mobile digits; the continue-link service uses it to find a returning customer's draft.</t>
         </is>
       </c>
     </row>
@@ -5827,7 +5899,7 @@
       <c r="J42" s="2" t="inlineStr"/>
       <c r="K42" s="2" t="inlineStr">
         <is>
-          <t>Internal key</t>
+          <t>Internal key.</t>
         </is>
       </c>
     </row>
@@ -5874,7 +5946,7 @@
       <c r="J43" s="2" t="inlineStr"/>
       <c r="K43" s="2" t="inlineStr">
         <is>
-          <t>Link to customers.id</t>
+          <t>Customer this address belongs to; links to customers.</t>
         </is>
       </c>
     </row>
@@ -5917,7 +5989,7 @@
       </c>
       <c r="K44" s="2" t="inlineStr">
         <is>
-          <t>Address type</t>
+          <t>PERMANENT | CURRENT | OFFICE. One row per type per customer.</t>
         </is>
       </c>
     </row>
@@ -5956,7 +6028,7 @@
       <c r="J45" s="2" t="inlineStr"/>
       <c r="K45" s="2" t="inlineStr">
         <is>
-          <t>Line1</t>
+          <t>First address line.</t>
         </is>
       </c>
     </row>
@@ -5995,7 +6067,7 @@
       <c r="J46" s="2" t="inlineStr"/>
       <c r="K46" s="2" t="inlineStr">
         <is>
-          <t>Line2</t>
+          <t>Second address line, optional.</t>
         </is>
       </c>
     </row>
@@ -6034,7 +6106,7 @@
       <c r="J47" s="2" t="inlineStr"/>
       <c r="K47" s="2" t="inlineStr">
         <is>
-          <t>City</t>
+          <t>City.</t>
         </is>
       </c>
     </row>
@@ -6073,7 +6145,7 @@
       <c r="J48" s="2" t="inlineStr"/>
       <c r="K48" s="2" t="inlineStr">
         <is>
-          <t>District</t>
+          <t>District, optional.</t>
         </is>
       </c>
     </row>
@@ -6120,7 +6192,7 @@
       <c r="J49" s="2" t="inlineStr"/>
       <c r="K49" s="2" t="inlineStr">
         <is>
-          <t>Link to states.code</t>
+          <t>State code; links to states.</t>
         </is>
       </c>
     </row>
@@ -6159,7 +6231,7 @@
       <c r="J50" s="2" t="inlineStr"/>
       <c r="K50" s="2" t="inlineStr">
         <is>
-          <t>Pincode</t>
+          <t>6-digit PIN code that cannot start with 0.</t>
         </is>
       </c>
     </row>
@@ -6202,7 +6274,7 @@
       <c r="J51" s="2" t="inlineStr"/>
       <c r="K51" s="2" t="inlineStr">
         <is>
-          <t>Source</t>
+          <t>Where the address came from: AADHAAR | EB_BILL | BUREAU | TYPED. Default TYPED.</t>
         </is>
       </c>
     </row>
@@ -6241,7 +6313,7 @@
       <c r="J52" s="2" t="inlineStr"/>
       <c r="K52" s="2" t="inlineStr">
         <is>
-          <t>Yes/no: rented</t>
+          <t>True when the current home is rented.</t>
         </is>
       </c>
     </row>
@@ -6280,7 +6352,7 @@
       <c r="J53" s="2" t="inlineStr"/>
       <c r="K53" s="2" t="inlineStr">
         <is>
-          <t>Owner name</t>
+          <t>House owner's name; required when the home is rented.</t>
         </is>
       </c>
     </row>
@@ -6319,7 +6391,7 @@
       <c r="J54" s="2" t="inlineStr"/>
       <c r="K54" s="2" t="inlineStr">
         <is>
-          <t>Owner contact</t>
+          <t>House owner's 10-digit mobile number; required when the home is rented.</t>
         </is>
       </c>
     </row>
@@ -6362,7 +6434,7 @@
       <c r="J55" s="2" t="inlineStr"/>
       <c r="K55" s="2" t="inlineStr">
         <is>
-          <t>Verified</t>
+          <t>Whether the address has been verified; set back to false whenever the customer saves it again.</t>
         </is>
       </c>
     </row>
@@ -6405,7 +6477,7 @@
       <c r="J56" s="2" t="inlineStr"/>
       <c r="K56" s="2" t="inlineStr">
         <is>
-          <t>When the row was created</t>
+          <t>When the row was created.</t>
         </is>
       </c>
     </row>
@@ -6444,7 +6516,7 @@
       <c r="J57" s="2" t="inlineStr"/>
       <c r="K57" s="2" t="inlineStr">
         <is>
-          <t>Years at address</t>
+          <t>Years lived at this address, 0 to 80.</t>
         </is>
       </c>
     </row>
@@ -6483,7 +6555,7 @@
       <c r="J58" s="2" t="inlineStr"/>
       <c r="K58" s="2" t="inlineStr">
         <is>
-          <t>Residence type</t>
+          <t>Type of home: OWNED | RENTED | FAMILY | COMPANY (checked by the address step, not by a database CHECK).</t>
         </is>
       </c>
     </row>
@@ -6530,7 +6602,7 @@
       <c r="J59" s="2" t="inlineStr"/>
       <c r="K59" s="2" t="inlineStr">
         <is>
-          <t>Internal key</t>
+          <t>Internal key.</t>
         </is>
       </c>
     </row>
@@ -6577,7 +6649,7 @@
       <c r="J60" s="2" t="inlineStr"/>
       <c r="K60" s="2" t="inlineStr">
         <is>
-          <t>Link to customers.id</t>
+          <t>Customer who gave the consent; links to customers.</t>
         </is>
       </c>
     </row>
@@ -6624,7 +6696,7 @@
       <c r="J61" s="2" t="inlineStr"/>
       <c r="K61" s="2" t="inlineStr">
         <is>
-          <t>Link to applications.id</t>
+          <t>Application the consent was given for; links to applications.</t>
         </is>
       </c>
     </row>
@@ -6671,7 +6743,7 @@
       <c r="J62" s="2" t="inlineStr"/>
       <c r="K62" s="2" t="inlineStr">
         <is>
-          <t>Link to consent_texts.purpose</t>
+          <t>What the consent covers, e.g. APPLICATION_PROCESSING or BUREAU_PULL. With version, points to consent_texts.</t>
         </is>
       </c>
     </row>
@@ -6718,7 +6790,7 @@
       <c r="J63" s="2" t="inlineStr"/>
       <c r="K63" s="2" t="inlineStr">
         <is>
-          <t>Link to consent_texts.version</t>
+          <t>Version of the wording accepted, e.g. 2026-09-v1. Only the current version can be accepted.</t>
         </is>
       </c>
     </row>
@@ -6757,7 +6829,7 @@
       <c r="J64" s="2" t="inlineStr"/>
       <c r="K64" s="2" t="inlineStr">
         <is>
-          <t>Body sha256</t>
+          <t>SHA-256 fingerprint of the exact wording shown, proving which text the customer accepted.</t>
         </is>
       </c>
     </row>
@@ -6796,7 +6868,7 @@
       <c r="J65" s="2" t="inlineStr"/>
       <c r="K65" s="2" t="inlineStr">
         <is>
-          <t>User agent</t>
+          <t>Browser details at the moment of consent, cut to 300 characters.</t>
         </is>
       </c>
     </row>
@@ -6839,7 +6911,7 @@
       <c r="J66" s="2" t="inlineStr"/>
       <c r="K66" s="2" t="inlineStr">
         <is>
-          <t>When given</t>
+          <t>When the consent was given.</t>
         </is>
       </c>
     </row>
@@ -6878,7 +6950,7 @@
       <c r="J67" s="2" t="inlineStr"/>
       <c r="K67" s="2" t="inlineStr">
         <is>
-          <t>When withdrawn</t>
+          <t>When the consent was withdrawn; empty while it still stands.</t>
         </is>
       </c>
     </row>
@@ -6921,7 +6993,7 @@
       <c r="J68" s="2" t="inlineStr"/>
       <c r="K68" s="2" t="inlineStr">
         <is>
-          <t>Purpose</t>
+          <t>What the consent covers: APPLICATION_PROCESSING or BUREAU_PULL in the seed. Part of the key with version.</t>
         </is>
       </c>
     </row>
@@ -6964,7 +7036,7 @@
       <c r="J69" s="2" t="inlineStr"/>
       <c r="K69" s="2" t="inlineStr">
         <is>
-          <t>Version</t>
+          <t>Version label of the wording, e.g. 2026-09-v1. Part of the key with purpose.</t>
         </is>
       </c>
     </row>
@@ -7003,7 +7075,7 @@
       <c r="J70" s="2" t="inlineStr"/>
       <c r="K70" s="2" t="inlineStr">
         <is>
-          <t>Body</t>
+          <t>Full consent wording shown to the customer.</t>
         </is>
       </c>
     </row>
@@ -7046,7 +7118,7 @@
       <c r="J71" s="2" t="inlineStr"/>
       <c r="K71" s="2" t="inlineStr">
         <is>
-          <t>Yes/no: current</t>
+          <t>True for the version customers can accept now; older versions stay for the record.</t>
         </is>
       </c>
     </row>
@@ -7089,7 +7161,7 @@
       <c r="J72" s="2" t="inlineStr"/>
       <c r="K72" s="2" t="inlineStr">
         <is>
-          <t>When the row was created</t>
+          <t>When the row was created.</t>
         </is>
       </c>
     </row>
@@ -7136,7 +7208,7 @@
       <c r="J73" s="2" t="inlineStr"/>
       <c r="K73" s="2" t="inlineStr">
         <is>
-          <t>Internal primary key</t>
+          <t>Internal key.</t>
         </is>
       </c>
     </row>
@@ -7179,7 +7251,7 @@
       <c r="J74" s="2" t="inlineStr"/>
       <c r="K74" s="2" t="inlineStr">
         <is>
-          <t>Public ID: YYYYMM + 6-digit serial (202608000001)</t>
+          <t>Readable reference: year and month (YYYYMM) plus a 6-digit serial number; unique.</t>
         </is>
       </c>
     </row>
@@ -7226,7 +7298,7 @@
       <c r="J75" s="2" t="inlineStr"/>
       <c r="K75" s="2" t="inlineStr">
         <is>
-          <t>Link to customer record</t>
+          <t>Applicant; links to customers.</t>
         </is>
       </c>
     </row>
@@ -7273,7 +7345,7 @@
       <c r="J76" s="2" t="inlineStr"/>
       <c r="K76" s="2" t="inlineStr">
         <is>
-          <t>Link to vehicle record; set at Step 2</t>
+          <t>Vehicle record for this application; links to vehicles.</t>
         </is>
       </c>
     </row>
@@ -7316,7 +7388,7 @@
       <c r="J77" s="2" t="inlineStr"/>
       <c r="K77" s="2" t="inlineStr">
         <is>
-          <t>DRAFT | IN_PRINCIPLE_APPROVED | DOCUMENTS_SUBMITTED | UNDER_ASSESSMENT | APPROVED | REJECTED | UNDER_REVIEW</t>
+          <t>Where the case stands; default DRAFT. Values used include SUBMITTED, UNDER_ASSESSMENT, UNDER_REVIEW, APPROVED, REJECTED, WITHDRAWN, CANCELLED, DISBURSED.</t>
         </is>
       </c>
     </row>
@@ -7359,7 +7431,7 @@
       <c r="J78" s="2" t="inlineStr"/>
       <c r="K78" s="2" t="inlineStr">
         <is>
-          <t>Last completed step (1-7)</t>
+          <t>Step reached in the staff application form; starts at 1.</t>
         </is>
       </c>
     </row>
@@ -7398,7 +7470,7 @@
       <c r="J79" s="2" t="inlineStr"/>
       <c r="K79" s="2" t="inlineStr">
         <is>
-          <t>On-road price minus down payment (Step 2)</t>
+          <t>Loan amount asked for, in INR.</t>
         </is>
       </c>
     </row>
@@ -7437,7 +7509,7 @@
       <c r="J80" s="2" t="inlineStr"/>
       <c r="K80" s="2" t="inlineStr">
         <is>
-          <t>Customer's own contribution</t>
+          <t>Customer's own payment towards the car, in INR.</t>
         </is>
       </c>
     </row>
@@ -7476,7 +7548,7 @@
       <c r="J81" s="2" t="inlineStr"/>
       <c r="K81" s="2" t="inlineStr">
         <is>
-          <t>Requested tenure in months (12-96)</t>
+          <t>Loan tenure, in months.</t>
         </is>
       </c>
     </row>
@@ -7515,7 +7587,7 @@
       <c r="J82" s="2" t="inlineStr"/>
       <c r="K82" s="2" t="inlineStr">
         <is>
-          <t>NEW | EXCHANGE | ADDITIONAL</t>
+          <t>Loan purpose, as a short code.</t>
         </is>
       </c>
     </row>
@@ -7554,7 +7626,7 @@
       <c r="J83" s="2" t="inlineStr"/>
       <c r="K83" s="2" t="inlineStr">
         <is>
-          <t>Make/model/year of current vehicle if exchange</t>
+          <t>Details of an old vehicle given in exchange, if any.</t>
         </is>
       </c>
     </row>
@@ -7593,7 +7665,7 @@
       <c r="J84" s="2" t="inlineStr"/>
       <c r="K84" s="2" t="inlineStr">
         <is>
-          <t>Does current vehicle have an outstanding loan?</t>
+          <t>Whether the exchanged vehicle still has a loan on it.</t>
         </is>
       </c>
     </row>
@@ -7632,7 +7704,7 @@
       <c r="J85" s="2" t="inlineStr"/>
       <c r="K85" s="2" t="inlineStr">
         <is>
-          <t>Outstanding loan on exchange vehicle</t>
+          <t>Amount still owed on the exchanged vehicle's loan, in INR.</t>
         </is>
       </c>
     </row>
@@ -7671,7 +7743,7 @@
       <c r="J86" s="2" t="inlineStr"/>
       <c r="K86" s="2" t="inlineStr">
         <is>
-          <t>Monthly EMI on exchange vehicle; feeds obligation</t>
+          <t>Monthly EMI on the exchanged vehicle's loan, in INR.</t>
         </is>
       </c>
     </row>
@@ -7710,7 +7782,7 @@
       <c r="J87" s="2" t="inlineStr"/>
       <c r="K87" s="2" t="inlineStr">
         <is>
-          <t>Self-declared monthly net salary (Step 3)</t>
+          <t>Net (take-home) monthly salary the customer declared, in INR.</t>
         </is>
       </c>
     </row>
@@ -7749,7 +7821,7 @@
       <c r="J88" s="2" t="inlineStr"/>
       <c r="K88" s="2" t="inlineStr">
         <is>
-          <t>Self-declared other monthly income</t>
+          <t>Other monthly income the customer declared, in INR.</t>
         </is>
       </c>
     </row>
@@ -7788,7 +7860,7 @@
       <c r="J89" s="2" t="inlineStr"/>
       <c r="K89" s="2" t="inlineStr">
         <is>
-          <t>Brief description of other income</t>
+          <t>Where the other income comes from, as the customer described it.</t>
         </is>
       </c>
     </row>
@@ -7827,7 +7899,7 @@
       <c r="J90" s="2" t="inlineStr"/>
       <c r="K90" s="2" t="inlineStr">
         <is>
-          <t>Self-declared total existing EMIs</t>
+          <t>Monthly EMIs the customer already pays, as declared, in INR.</t>
         </is>
       </c>
     </row>
@@ -7866,7 +7938,7 @@
       <c r="J91" s="2" t="inlineStr"/>
       <c r="K91" s="2" t="inlineStr">
         <is>
-          <t>Monthly rent/housing (0 if owned)</t>
+          <t>Monthly rent the customer declared, in INR.</t>
         </is>
       </c>
     </row>
@@ -7905,7 +7977,7 @@
       <c r="J92" s="2" t="inlineStr"/>
       <c r="K92" s="2" t="inlineStr">
         <is>
-          <t>Monthly insurance premiums</t>
+          <t>Monthly insurance premiums the customer declared, in INR.</t>
         </is>
       </c>
     </row>
@@ -7944,7 +8016,7 @@
       <c r="J93" s="2" t="inlineStr"/>
       <c r="K93" s="2" t="inlineStr">
         <is>
-          <t>Monthly food/household expenses</t>
+          <t>Monthly food and household spending the customer declared, in INR.</t>
         </is>
       </c>
     </row>
@@ -7983,7 +8055,7 @@
       <c r="J94" s="2" t="inlineStr"/>
       <c r="K94" s="2" t="inlineStr">
         <is>
-          <t>Monthly travel/commute</t>
+          <t>Monthly travel spending the customer declared, in INR.</t>
         </is>
       </c>
     </row>
@@ -8022,7 +8094,7 @@
       <c r="J95" s="2" t="inlineStr"/>
       <c r="K95" s="2" t="inlineStr">
         <is>
-          <t>Other regular monthly expenses</t>
+          <t>Other monthly expenses the customer declared, in INR.</t>
         </is>
       </c>
     </row>
@@ -8061,7 +8133,7 @@
       <c r="J96" s="2" t="inlineStr"/>
       <c r="K96" s="2" t="inlineStr">
         <is>
-          <t>System-calculated indicative EMI at Step 4</t>
+          <t>Monthly EMI worked out by the in-principle check, in INR.</t>
         </is>
       </c>
     </row>
@@ -8100,7 +8172,7 @@
       <c r="J97" s="2" t="inlineStr"/>
       <c r="K97" s="2" t="inlineStr">
         <is>
-          <t>Rate shown at in-principle stage</t>
+          <t>Interest rate from the rate grid used in the in-principle check, % per year.</t>
         </is>
       </c>
     </row>
@@ -8139,7 +8211,7 @@
       <c r="J98" s="2" t="inlineStr"/>
       <c r="K98" s="2" t="inlineStr">
         <is>
-          <t>ELIGIBLE | NOT_ELIGIBLE (Step 4 quick check)</t>
+          <t>Outcome of the in-principle check: ELIGIBLE | NOT_ELIGIBLE.</t>
         </is>
       </c>
     </row>
@@ -8178,7 +8250,7 @@
       <c r="J99" s="2" t="inlineStr"/>
       <c r="K99" s="2" t="inlineStr">
         <is>
-          <t>When in-principle decision was made</t>
+          <t>When the in-principle check ran.</t>
         </is>
       </c>
     </row>
@@ -8217,7 +8289,7 @@
       <c r="J100" s="2" t="inlineStr"/>
       <c r="K100" s="2" t="inlineStr">
         <is>
-          <t>When all 9 docs uploaded</t>
+          <t>When the documents were submitted; filled at customer submit if not already set.</t>
         </is>
       </c>
     </row>
@@ -8256,7 +8328,7 @@
       <c r="J101" s="2" t="inlineStr"/>
       <c r="K101" s="2" t="inlineStr">
         <is>
-          <t>When Step 7 assessment began</t>
+          <t>When the credit assessment started.</t>
         </is>
       </c>
     </row>
@@ -8295,7 +8367,7 @@
       <c r="J102" s="2" t="inlineStr"/>
       <c r="K102" s="2" t="inlineStr">
         <is>
-          <t>When final decision was recorded</t>
+          <t>When the final credit decision was recorded.</t>
         </is>
       </c>
     </row>
@@ -8334,7 +8406,7 @@
       <c r="J103" s="2" t="inlineStr"/>
       <c r="K103" s="2" t="inlineStr">
         <is>
-          <t>Draft auto-expires 15 days after creation</t>
+          <t>When an unfinished draft expires.</t>
         </is>
       </c>
     </row>
@@ -8373,7 +8445,7 @@
       <c r="J104" s="2" t="inlineStr"/>
       <c r="K104" s="2" t="inlineStr">
         <is>
-          <t>Sanction letter valid for 30 calendar days</t>
+          <t>Date and time until which the sanction stays valid.</t>
         </is>
       </c>
     </row>
@@ -8420,7 +8492,7 @@
       <c r="J105" s="2" t="inlineStr"/>
       <c r="K105" s="2" t="inlineStr">
         <is>
-          <t>Credit officer assigned for Maybe cases</t>
+          <t>Staff user handling the case; links to users.</t>
         </is>
       </c>
     </row>
@@ -8467,7 +8539,7 @@
       <c r="J106" s="2" t="inlineStr"/>
       <c r="K106" s="2" t="inlineStr">
         <is>
-          <t>State where vehicle will be registered</t>
+          <t>State the application belongs to; links to states.</t>
         </is>
       </c>
     </row>
@@ -8510,7 +8582,7 @@
       <c r="J107" s="2" t="inlineStr"/>
       <c r="K107" s="2" t="inlineStr">
         <is>
-          <t>Record creation timestamp</t>
+          <t>When the row was created.</t>
         </is>
       </c>
     </row>
@@ -8553,7 +8625,7 @@
       <c r="J108" s="2" t="inlineStr"/>
       <c r="K108" s="2" t="inlineStr">
         <is>
-          <t>Last update timestamp</t>
+          <t>When the row was last changed; set automatically.</t>
         </is>
       </c>
     </row>
@@ -8596,7 +8668,7 @@
       <c r="J109" s="2" t="inlineStr"/>
       <c r="K109" s="2" t="inlineStr">
         <is>
-          <t>Channel</t>
+          <t>Lead channel the application came through; default DIRECT.</t>
         </is>
       </c>
     </row>
@@ -8639,7 +8711,7 @@
       <c r="J110" s="2" t="inlineStr"/>
       <c r="K110" s="2" t="inlineStr">
         <is>
-          <t>Onboarding step</t>
+          <t>Customer journey step reached: 1 sign-up, 2 car details, 3 documents, 4 personal/address/work details, 5 submitted.</t>
         </is>
       </c>
     </row>
@@ -8678,7 +8750,7 @@
       <c r="J111" s="2" t="inlineStr"/>
       <c r="K111" s="2" t="inlineStr">
         <is>
-          <t>Approval stage</t>
+          <t>IN_PRINCIPLE | FINAL. Set at submit: FINAL if the dealer quotation is in, otherwise IN_PRINCIPLE.</t>
         </is>
       </c>
     </row>
@@ -8721,7 +8793,7 @@
       <c r="J112" s="2" t="inlineStr"/>
       <c r="K112" s="2" t="inlineStr">
         <is>
-          <t>Quote pending</t>
+          <t>True when car details were typed in, so the dealer quotation is still owed before final approval.</t>
         </is>
       </c>
     </row>
@@ -8760,7 +8832,7 @@
       <c r="J113" s="2" t="inlineStr"/>
       <c r="K113" s="2" t="inlineStr">
         <is>
-          <t>When customer submitted</t>
+          <t>When the customer submitted the application.</t>
         </is>
       </c>
     </row>
@@ -8803,7 +8875,7 @@
       <c r="J114" s="2" t="inlineStr"/>
       <c r="K114" s="2" t="inlineStr">
         <is>
-          <t>Origin</t>
+          <t>STAFF | CUSTOMER. Default STAFF; set to CUSTOMER automatically when the case gets a document checklist (customer journey).</t>
         </is>
       </c>
     </row>
@@ -8842,7 +8914,7 @@
       <c r="J115" s="2" t="inlineStr"/>
       <c r="K115" s="2" t="inlineStr">
         <is>
-          <t>Auto review</t>
+          <t>Latest automatic document review summary (JSON): documents accepted, asked again, still reading, engine recommendation, fast-lane flag. Written by the engine.</t>
         </is>
       </c>
     </row>
@@ -8889,7 +8961,7 @@
       <c r="J116" s="2" t="inlineStr"/>
       <c r="K116" s="2" t="inlineStr">
         <is>
-          <t>Link to employers.id</t>
+          <t>Employer Master record this case was matched to; links to employers, cleared if that employer is deleted.</t>
         </is>
       </c>
     </row>
@@ -8928,7 +9000,7 @@
       <c r="J117" s="2" t="inlineStr"/>
       <c r="K117" s="2" t="inlineStr">
         <is>
-          <t>Employer category</t>
+          <t>Employer category A | B | C used to price this case. Written by the engine.</t>
         </is>
       </c>
     </row>
@@ -8967,7 +9039,7 @@
       <c r="J118" s="2" t="inlineStr"/>
       <c r="K118" s="2" t="inlineStr">
         <is>
-          <t>Employer category basis</t>
+          <t>How the category was set: MASTER_VERIFIED | MASTER_PROVISIONAL | DECLARED_TYPE (from the type the customer gave).</t>
         </is>
       </c>
     </row>
@@ -9014,7 +9086,7 @@
       <c r="J119" s="2" t="inlineStr"/>
       <c r="K119" s="2" t="inlineStr">
         <is>
-          <t>Link to applications.id</t>
+          <t>Application these details belong to; links to applications. Part of the key.</t>
         </is>
       </c>
     </row>
@@ -9061,7 +9133,7 @@
       </c>
       <c r="K120" s="2" t="inlineStr">
         <is>
-          <t>Group code</t>
+          <t>Which group of details: PERSONAL | ADDRESS | EMPLOYMENT. Part of the key.</t>
         </is>
       </c>
     </row>
@@ -9104,7 +9176,7 @@
       <c r="J121" s="2" t="inlineStr"/>
       <c r="K121" s="2" t="inlineStr">
         <is>
-          <t>Prefilled</t>
+          <t>What the system showed the customer, read from the documents (JSON).</t>
         </is>
       </c>
     </row>
@@ -9143,7 +9215,7 @@
       <c r="J122" s="2" t="inlineStr"/>
       <c r="K122" s="2" t="inlineStr">
         <is>
-          <t>Confirmed</t>
+          <t>What the customer confirmed (JSON).</t>
         </is>
       </c>
     </row>
@@ -9186,7 +9258,7 @@
       <c r="J123" s="2" t="inlineStr"/>
       <c r="K123" s="2" t="inlineStr">
         <is>
-          <t>Edited fields</t>
+          <t>Names of pre-filled fields the customer changed; a signal for the manual-edit checks.</t>
         </is>
       </c>
     </row>
@@ -9229,7 +9301,7 @@
       <c r="J124" s="2" t="inlineStr"/>
       <c r="K124" s="2" t="inlineStr">
         <is>
-          <t>When confirmed</t>
+          <t>When the customer last confirmed this group.</t>
         </is>
       </c>
     </row>
@@ -9276,7 +9348,7 @@
       <c r="J125" s="2" t="inlineStr"/>
       <c r="K125" s="2" t="inlineStr">
         <is>
-          <t>Internal key</t>
+          <t>Internal key.</t>
         </is>
       </c>
     </row>
@@ -9323,7 +9395,7 @@
       <c r="J126" s="2" t="inlineStr"/>
       <c r="K126" s="2" t="inlineStr">
         <is>
-          <t>Link to applications.id</t>
+          <t>Application the event belongs to; links to applications.</t>
         </is>
       </c>
     </row>
@@ -9362,7 +9434,7 @@
       <c r="J127" s="2" t="inlineStr"/>
       <c r="K127" s="2" t="inlineStr">
         <is>
-          <t>Stage</t>
+          <t>Stage reached. Values used: RECEIVED, DOCS_VERIFIED, CREDIT_CHECK, DECISION, KFS_ACCEPTED, AGREEMENT_SIGNED, DISBURSED.</t>
         </is>
       </c>
     </row>
@@ -9401,7 +9473,7 @@
       <c r="J128" s="2" t="inlineStr"/>
       <c r="K128" s="2" t="inlineStr">
         <is>
-          <t>Note</t>
+          <t>Short message for the customer, e.g. "Submitted by the customer".</t>
         </is>
       </c>
     </row>
@@ -9444,7 +9516,7 @@
       <c r="J129" s="2" t="inlineStr"/>
       <c r="K129" s="2" t="inlineStr">
         <is>
-          <t>At</t>
+          <t>When the stage was reached.</t>
         </is>
       </c>
     </row>
@@ -9491,7 +9563,7 @@
       <c r="J130" s="2" t="inlineStr"/>
       <c r="K130" s="2" t="inlineStr">
         <is>
-          <t>Link to applications.id</t>
+          <t>Application this checklist line belongs to; links to applications. Part of the key.</t>
         </is>
       </c>
     </row>
@@ -9538,7 +9610,7 @@
       <c r="J131" s="2" t="inlineStr"/>
       <c r="K131" s="2" t="inlineStr">
         <is>
-          <t>Link to document_types.code</t>
+          <t>Document code from document_types, e.g. PAN, AADHAAR, SALARY_SLIP, FORM16_B, BANK_STMT, QUOTE, EB_BILL. Part of the key.</t>
         </is>
       </c>
     </row>
@@ -9577,7 +9649,7 @@
       <c r="J132" s="2" t="inlineStr"/>
       <c r="K132" s="2" t="inlineStr">
         <is>
-          <t>Required</t>
+          <t>ALWAYS | CONDITIONAL | OPTIONAL, copied from document_types. EB_BILL becomes ALWAYS when the current address differs from the permanent one.</t>
         </is>
       </c>
     </row>
@@ -9624,7 +9696,7 @@
       </c>
       <c r="K133" s="2" t="inlineStr">
         <is>
-          <t>Status</t>
+          <t>MISSING | RECEIVED | ACCEPTED | REUPLOAD | WAIVED | NOT_NEEDED. Default MISSING. Submit needs every ALWAYS document received, accepted or waived.</t>
         </is>
       </c>
     </row>
@@ -9663,7 +9735,7 @@
       <c r="J134" s="2" t="inlineStr"/>
       <c r="K134" s="2" t="inlineStr">
         <is>
-          <t>Reason</t>
+          <t>Note to the customer: what to upload, or why a document is asked for again.</t>
         </is>
       </c>
     </row>
@@ -9706,7 +9778,7 @@
       <c r="J135" s="2" t="inlineStr"/>
       <c r="K135" s="2" t="inlineStr">
         <is>
-          <t>When the row was last changed</t>
+          <t>When the row was last changed.</t>
         </is>
       </c>
     </row>
@@ -9753,7 +9825,7 @@
       <c r="J136" s="2" t="inlineStr"/>
       <c r="K136" s="2" t="inlineStr">
         <is>
-          <t>Internal primary key</t>
+          <t>Internal key.</t>
         </is>
       </c>
     </row>
@@ -9800,7 +9872,7 @@
       <c r="J137" s="2" t="inlineStr"/>
       <c r="K137" s="2" t="inlineStr">
         <is>
-          <t>Link to application</t>
+          <t>Application this vehicle is for; links to applications.</t>
         </is>
       </c>
     </row>
@@ -9839,7 +9911,7 @@
       <c r="J138" s="2" t="inlineStr"/>
       <c r="K138" s="2" t="inlineStr">
         <is>
-          <t>Vehicle manufacturer/brand</t>
+          <t>Car brand, e.g. Hyundai.</t>
         </is>
       </c>
     </row>
@@ -9878,7 +9950,7 @@
       <c r="J139" s="2" t="inlineStr"/>
       <c r="K139" s="2" t="inlineStr">
         <is>
-          <t>Vehicle model name</t>
+          <t>Car model.</t>
         </is>
       </c>
     </row>
@@ -9917,7 +9989,7 @@
       <c r="J140" s="2" t="inlineStr"/>
       <c r="K140" s="2" t="inlineStr">
         <is>
-          <t>Variant/trim level</t>
+          <t>Model variant or trim.</t>
         </is>
       </c>
     </row>
@@ -9956,7 +10028,7 @@
       <c r="J141" s="2" t="inlineStr"/>
       <c r="K141" s="2" t="inlineStr">
         <is>
-          <t>PETROL | DIESEL | CNG | HYBRID | ELECTRIC</t>
+          <t>Fuel type of the car.</t>
         </is>
       </c>
     </row>
@@ -9995,7 +10067,7 @@
       <c r="J142" s="2" t="inlineStr"/>
       <c r="K142" s="2" t="inlineStr">
         <is>
-          <t>CAR | SCV | LCV | 3W (Phase 1: CAR only)</t>
+          <t>Vehicle segment code; the engine prices on CAR (Phase 1 is cars only).</t>
         </is>
       </c>
     </row>
@@ -10034,7 +10106,7 @@
       <c r="J143" s="2" t="inlineStr"/>
       <c r="K143" s="2" t="inlineStr">
         <is>
-          <t>Ex-showroom price (LTV base)</t>
+          <t>Ex-showroom price, in INR.</t>
         </is>
       </c>
     </row>
@@ -10073,7 +10145,7 @@
       <c r="J144" s="2" t="inlineStr"/>
       <c r="K144" s="2" t="inlineStr">
         <is>
-          <t>Road tax amount</t>
+          <t>Road tax, in INR.</t>
         </is>
       </c>
     </row>
@@ -10112,7 +10184,7 @@
       <c r="J145" s="2" t="inlineStr"/>
       <c r="K145" s="2" t="inlineStr">
         <is>
-          <t>First-year insurance premium</t>
+          <t>Insurance cost, in INR.</t>
         </is>
       </c>
     </row>
@@ -10151,7 +10223,7 @@
       <c r="J146" s="2" t="inlineStr"/>
       <c r="K146" s="2" t="inlineStr">
         <is>
-          <t>Registration + other charges</t>
+          <t>Registration charges, in INR.</t>
         </is>
       </c>
     </row>
@@ -10190,7 +10262,7 @@
       <c r="J147" s="2" t="inlineStr"/>
       <c r="K147" s="2" t="inlineStr">
         <is>
-          <t>Calculated: ex_showroom + tax + insurance + reg</t>
+          <t>Total on-road price, in INR.</t>
         </is>
       </c>
     </row>
@@ -10237,7 +10309,7 @@
       <c r="J148" s="2" t="inlineStr"/>
       <c r="K148" s="2" t="inlineStr">
         <is>
-          <t>Dealer (Phase 2; null in Phase 1 direct)</t>
+          <t>Dealer selling the car; links to dealers.</t>
         </is>
       </c>
     </row>
@@ -10276,7 +10348,7 @@
       <c r="J149" s="2" t="inlineStr"/>
       <c r="K149" s="2" t="inlineStr">
         <is>
-          <t>Dealer proforma invoice number</t>
+          <t>Dealer quotation number.</t>
         </is>
       </c>
     </row>
@@ -10315,7 +10387,7 @@
       <c r="J150" s="2" t="inlineStr"/>
       <c r="K150" s="2" t="inlineStr">
         <is>
-          <t>Date on dealer quotation</t>
+          <t>Date on the dealer quotation.</t>
         </is>
       </c>
     </row>
@@ -10358,7 +10430,7 @@
       <c r="J151" s="2" t="inlineStr"/>
       <c r="K151" s="2" t="inlineStr">
         <is>
-          <t>True if quotation matches Step 2 data</t>
+          <t>Whether the dealer quotation has been verified; default false.</t>
         </is>
       </c>
     </row>
@@ -10401,7 +10473,7 @@
       <c r="J152" s="2" t="inlineStr"/>
       <c r="K152" s="2" t="inlineStr">
         <is>
-          <t>Record creation timestamp</t>
+          <t>When the row was created.</t>
         </is>
       </c>
     </row>
@@ -10444,7 +10516,7 @@
       <c r="J153" s="2" t="inlineStr"/>
       <c r="K153" s="2" t="inlineStr">
         <is>
-          <t>Last update timestamp</t>
+          <t>When the row was last changed; set automatically.</t>
         </is>
       </c>
     </row>
@@ -10491,7 +10563,7 @@
       <c r="J154" s="2" t="inlineStr"/>
       <c r="K154" s="2" t="inlineStr">
         <is>
-          <t>Internal key</t>
+          <t>Internal key.</t>
         </is>
       </c>
     </row>
@@ -10538,7 +10610,7 @@
       <c r="J155" s="2" t="inlineStr"/>
       <c r="K155" s="2" t="inlineStr">
         <is>
-          <t>Link to applications.id</t>
+          <t>Application this quotation is for; one quotation per application.</t>
         </is>
       </c>
     </row>
@@ -10581,7 +10653,7 @@
       </c>
       <c r="K156" s="2" t="inlineStr">
         <is>
-          <t>Source</t>
+          <t>QUOTATION | MANUAL. MANUAL (typed in) means the dealer quotation is still owed before final approval.</t>
         </is>
       </c>
     </row>
@@ -10628,7 +10700,7 @@
       <c r="J157" s="2" t="inlineStr"/>
       <c r="K157" s="2" t="inlineStr">
         <is>
-          <t>Link to documents.id</t>
+          <t>Uploaded quotation file; links to documents.</t>
         </is>
       </c>
     </row>
@@ -10667,7 +10739,7 @@
       <c r="J158" s="2" t="inlineStr"/>
       <c r="K158" s="2" t="inlineStr">
         <is>
-          <t>Customer name on quote</t>
+          <t>Customer name as printed on the quotation.</t>
         </is>
       </c>
     </row>
@@ -10706,7 +10778,7 @@
       <c r="J159" s="2" t="inlineStr"/>
       <c r="K159" s="2" t="inlineStr">
         <is>
-          <t>Name match pct</t>
+          <t>How closely the name on the quote matches the customer's name, in %.</t>
         </is>
       </c>
     </row>
@@ -10753,7 +10825,7 @@
       <c r="J160" s="2" t="inlineStr"/>
       <c r="K160" s="2" t="inlineStr">
         <is>
-          <t>Link to dealers.id</t>
+          <t>Dealer matched by exact name (case ignored); links to dealers. Empty if no match.</t>
         </is>
       </c>
     </row>
@@ -10792,7 +10864,7 @@
       <c r="J161" s="2" t="inlineStr"/>
       <c r="K161" s="2" t="inlineStr">
         <is>
-          <t>Dealer name</t>
+          <t>Dealer name as entered.</t>
         </is>
       </c>
     </row>
@@ -10831,7 +10903,7 @@
       <c r="J162" s="2" t="inlineStr"/>
       <c r="K162" s="2" t="inlineStr">
         <is>
-          <t>Sales officer name</t>
+          <t>Dealer's sales officer name.</t>
         </is>
       </c>
     </row>
@@ -10870,7 +10942,7 @@
       <c r="J163" s="2" t="inlineStr"/>
       <c r="K163" s="2" t="inlineStr">
         <is>
-          <t>Sales officer mobile</t>
+          <t>Sales officer's 10-digit mobile number, stored as digits only.</t>
         </is>
       </c>
     </row>
@@ -10909,7 +10981,7 @@
       <c r="J164" s="2" t="inlineStr"/>
       <c r="K164" s="2" t="inlineStr">
         <is>
-          <t>Quote date</t>
+          <t>Date of the quotation; required for a QUOTATION and cannot be in the future.</t>
         </is>
       </c>
     </row>
@@ -10948,7 +11020,7 @@
       <c r="J165" s="2" t="inlineStr"/>
       <c r="K165" s="2" t="inlineStr">
         <is>
-          <t>Valid until</t>
+          <t>Last valid date of the quotation; an expired quote is refused.</t>
         </is>
       </c>
     </row>
@@ -10987,7 +11059,7 @@
       <c r="J166" s="2" t="inlineStr"/>
       <c r="K166" s="2" t="inlineStr">
         <is>
-          <t>Make</t>
+          <t>Car brand.</t>
         </is>
       </c>
     </row>
@@ -11026,7 +11098,7 @@
       <c r="J167" s="2" t="inlineStr"/>
       <c r="K167" s="2" t="inlineStr">
         <is>
-          <t>Model</t>
+          <t>Car model.</t>
         </is>
       </c>
     </row>
@@ -11065,7 +11137,7 @@
       <c r="J168" s="2" t="inlineStr"/>
       <c r="K168" s="2" t="inlineStr">
         <is>
-          <t>Variant</t>
+          <t>Model variant, optional.</t>
         </is>
       </c>
     </row>
@@ -11104,7 +11176,7 @@
       <c r="J169" s="2" t="inlineStr"/>
       <c r="K169" s="2" t="inlineStr">
         <is>
-          <t>Colour</t>
+          <t>Car colour, optional.</t>
         </is>
       </c>
     </row>
@@ -11143,7 +11215,7 @@
       <c r="J170" s="2" t="inlineStr"/>
       <c r="K170" s="2" t="inlineStr">
         <is>
-          <t>Fuel type</t>
+          <t>PETROL | DIESEL | CNG | EV | HYBRID, or empty.</t>
         </is>
       </c>
     </row>
@@ -11182,7 +11254,7 @@
       <c r="J171" s="2" t="inlineStr"/>
       <c r="K171" s="2" t="inlineStr">
         <is>
-          <t>Ex showroom</t>
+          <t>Ex-showroom price in INR; must be above 0, and the form accepts ₹1 lakh to ₹2 crore.</t>
         </is>
       </c>
     </row>
@@ -11221,7 +11293,7 @@
       <c r="J172" s="2" t="inlineStr"/>
       <c r="K172" s="2" t="inlineStr">
         <is>
-          <t>Road tax</t>
+          <t>Road tax, in INR.</t>
         </is>
       </c>
     </row>
@@ -11260,7 +11332,7 @@
       <c r="J173" s="2" t="inlineStr"/>
       <c r="K173" s="2" t="inlineStr">
         <is>
-          <t>Insurance</t>
+          <t>Insurance cost, in INR.</t>
         </is>
       </c>
     </row>
@@ -11299,7 +11371,7 @@
       <c r="J174" s="2" t="inlineStr"/>
       <c r="K174" s="2" t="inlineStr">
         <is>
-          <t>On road</t>
+          <t>On-road price in INR, worked out as ex-showroom plus road tax plus insurance.</t>
         </is>
       </c>
     </row>
@@ -11338,7 +11410,7 @@
       <c r="J175" s="2" t="inlineStr"/>
       <c r="K175" s="2" t="inlineStr">
         <is>
-          <t>Loan amount requested</t>
+          <t>Loan asked for in INR; at least ₹1 lakh and not above the on-road price.</t>
         </is>
       </c>
     </row>
@@ -11377,7 +11449,7 @@
       <c r="J176" s="2" t="inlineStr"/>
       <c r="K176" s="2" t="inlineStr">
         <is>
-          <t>Tenure months</t>
+          <t>Loan tenure in months. CHECK allows 12 to 96; the form accepts 24 | 36 | 48 | 60 | 72 | 84.</t>
         </is>
       </c>
     </row>
@@ -11420,7 +11492,7 @@
       <c r="J177" s="2" t="inlineStr"/>
       <c r="K177" s="2" t="inlineStr">
         <is>
-          <t>When the row was created</t>
+          <t>When the row was created.</t>
         </is>
       </c>
     </row>
@@ -11463,7 +11535,7 @@
       <c r="J178" s="2" t="inlineStr"/>
       <c r="K178" s="2" t="inlineStr">
         <is>
-          <t>When the row was last changed</t>
+          <t>When the row was last changed.</t>
         </is>
       </c>
     </row>
@@ -11510,7 +11582,7 @@
       <c r="J179" s="2" t="inlineStr"/>
       <c r="K179" s="2" t="inlineStr">
         <is>
-          <t>Internal primary key</t>
+          <t>Internal key.</t>
         </is>
       </c>
     </row>
@@ -11553,7 +11625,7 @@
       <c r="J180" s="2" t="inlineStr"/>
       <c r="K180" s="2" t="inlineStr">
         <is>
-          <t>Unique dealer identifier</t>
+          <t>Unique dealer code, e.g. HYD-DEL-001 (make, city, serial).</t>
         </is>
       </c>
     </row>
@@ -11592,7 +11664,7 @@
       <c r="J181" s="2" t="inlineStr"/>
       <c r="K181" s="2" t="inlineStr">
         <is>
-          <t>Dealer firm name</t>
+          <t>Dealership name.</t>
         </is>
       </c>
     </row>
@@ -11631,7 +11703,7 @@
       <c r="J182" s="2" t="inlineStr"/>
       <c r="K182" s="2" t="inlineStr">
         <is>
-          <t>OEM/brand the dealer represents</t>
+          <t>Car brand the dealer sells.</t>
         </is>
       </c>
     </row>
@@ -11670,7 +11742,7 @@
       <c r="J183" s="2" t="inlineStr"/>
       <c r="K183" s="2" t="inlineStr">
         <is>
-          <t>Dealer city</t>
+          <t>City of the dealership.</t>
         </is>
       </c>
     </row>
@@ -11717,7 +11789,7 @@
       <c r="J184" s="2" t="inlineStr"/>
       <c r="K184" s="2" t="inlineStr">
         <is>
-          <t>State code</t>
+          <t>State of the dealership; links to states.</t>
         </is>
       </c>
     </row>
@@ -11756,7 +11828,7 @@
       <c r="J185" s="2" t="inlineStr"/>
       <c r="K185" s="2" t="inlineStr">
         <is>
-          <t>LOW | MEDIUM | HIGH (Phase 2 dealer scoring)</t>
+          <t>Dealer risk tier label; not set in the seed data.</t>
         </is>
       </c>
     </row>
@@ -11799,7 +11871,7 @@
       <c r="J186" s="2" t="inlineStr"/>
       <c r="K186" s="2" t="inlineStr">
         <is>
-          <t>Active dealer flag</t>
+          <t>Whether the dealer is currently active; default true.</t>
         </is>
       </c>
     </row>
@@ -11842,7 +11914,7 @@
       <c r="J187" s="2" t="inlineStr"/>
       <c r="K187" s="2" t="inlineStr">
         <is>
-          <t>Record creation timestamp</t>
+          <t>When the row was created.</t>
         </is>
       </c>
     </row>
@@ -11885,7 +11957,7 @@
       <c r="J188" s="2" t="inlineStr"/>
       <c r="K188" s="2" t="inlineStr">
         <is>
-          <t>Last update timestamp</t>
+          <t>When the row was last changed; set automatically.</t>
         </is>
       </c>
     </row>
@@ -11928,7 +12000,7 @@
       <c r="J189" s="2" t="inlineStr"/>
       <c r="K189" s="2" t="inlineStr">
         <is>
-          <t>State abbreviation code</t>
+          <t>Short state code, e.g. AP; the key.</t>
         </is>
       </c>
     </row>
@@ -11971,7 +12043,7 @@
       <c r="J190" s="2" t="inlineStr"/>
       <c r="K190" s="2" t="inlineStr">
         <is>
-          <t>Full state name</t>
+          <t>Full state name; unique.</t>
         </is>
       </c>
     </row>
@@ -12014,7 +12086,7 @@
       <c r="J191" s="2" t="inlineStr"/>
       <c r="K191" s="2" t="inlineStr">
         <is>
-          <t>Whether lending operations active in this state</t>
+          <t>Whether the lender operates in this state; default true.</t>
         </is>
       </c>
     </row>
@@ -12053,7 +12125,7 @@
       <c r="J192" s="2" t="inlineStr"/>
       <c r="K192" s="2" t="inlineStr">
         <is>
-          <t>Default road tax % for the state (reference)</t>
+          <t>State road tax rate, in %; empty for states where the lender does not operate.</t>
         </is>
       </c>
     </row>
@@ -12096,7 +12168,7 @@
       <c r="J193" s="2" t="inlineStr"/>
       <c r="K193" s="2" t="inlineStr">
         <is>
-          <t>Record creation timestamp</t>
+          <t>When the row was created.</t>
         </is>
       </c>
     </row>
@@ -28389,7 +28461,7 @@
       <c r="J592" s="2" t="inlineStr"/>
       <c r="K592" s="2" t="inlineStr">
         <is>
-          <t>Internal key</t>
+          <t>Internal key.</t>
         </is>
       </c>
     </row>
@@ -28428,7 +28500,7 @@
       <c r="J593" s="2" t="inlineStr"/>
       <c r="K593" s="2" t="inlineStr">
         <is>
-          <t>Name</t>
+          <t>Employer's name.</t>
         </is>
       </c>
     </row>
@@ -28471,7 +28543,7 @@
       <c r="J594" s="2" t="inlineStr"/>
       <c r="K594" s="2" t="inlineStr">
         <is>
-          <t>Name key</t>
+          <t>Name in lower case with Ltd, Pvt, India and similar words removed, so spelling variants match; unique.</t>
         </is>
       </c>
     </row>
@@ -28514,7 +28586,7 @@
       <c r="J595" s="2" t="inlineStr"/>
       <c r="K595" s="2" t="inlineStr">
         <is>
-          <t>Aliases</t>
+          <t>Other names the employer appears under on payslips and Form 16.</t>
         </is>
       </c>
     </row>
@@ -28553,7 +28625,7 @@
       <c r="J596" s="2" t="inlineStr"/>
       <c r="K596" s="2" t="inlineStr">
         <is>
-          <t>Cin</t>
+          <t>Company Identification Number in the 21-character MCA format, starting L (listed) or U (unlisted).</t>
         </is>
       </c>
     </row>
@@ -28592,7 +28664,7 @@
       <c r="J597" s="2" t="inlineStr"/>
       <c r="K597" s="2" t="inlineStr">
         <is>
-          <t>Gstin</t>
+          <t>GST number, 15 characters; the checks test its format and check character.</t>
         </is>
       </c>
     </row>
@@ -28639,7 +28711,7 @@
       </c>
       <c r="K598" s="2" t="inlineStr">
         <is>
-          <t>Employer type</t>
+          <t>GOVERNMENT | PSU | LISTED | MNC | PUBLIC_LTD | PRIVATE_LTD | LLP | PARTNERSHIP | PROPRIETORSHIP | OTHER. Default OTHER.</t>
         </is>
       </c>
     </row>
@@ -28686,7 +28758,7 @@
       </c>
       <c r="K599" s="2" t="inlineStr">
         <is>
-          <t>Category</t>
+          <t>A | B | C, default C. Set by rule when added; changed later only by an approved category change.</t>
         </is>
       </c>
     </row>
@@ -28729,7 +28801,7 @@
       <c r="J600" s="2" t="inlineStr"/>
       <c r="K600" s="2" t="inlineStr">
         <is>
-          <t>Verified</t>
+          <t>True only when no latest check is FAIL or REVIEW; until then the category is provisional. Any edit sets it back to false.</t>
         </is>
       </c>
     </row>
@@ -28768,7 +28840,7 @@
       <c r="J601" s="2" t="inlineStr"/>
       <c r="K601" s="2" t="inlineStr">
         <is>
-          <t>Listed</t>
+          <t>Whether listed on NSE/BSE; set by the checks (on the listed list or CIN starts with L).</t>
         </is>
       </c>
     </row>
@@ -28807,7 +28879,7 @@
       <c r="J602" s="2" t="inlineStr"/>
       <c r="K602" s="2" t="inlineStr">
         <is>
-          <t>Listed symbol</t>
+          <t>Stock symbol from the listed-company list.</t>
         </is>
       </c>
     </row>
@@ -28846,7 +28918,7 @@
       <c r="J603" s="2" t="inlineStr"/>
       <c r="K603" s="2" t="inlineStr">
         <is>
-          <t>Incorporation year</t>
+          <t>Year the company was incorporated; set by the checks.</t>
         </is>
       </c>
     </row>
@@ -28885,7 +28957,7 @@
       <c r="J604" s="2" t="inlineStr"/>
       <c r="K604" s="2" t="inlineStr">
         <is>
-          <t>Incorporated on</t>
+          <t>Exact incorporation date, if known.</t>
         </is>
       </c>
     </row>
@@ -28924,7 +28996,7 @@
       <c r="J605" s="2" t="inlineStr"/>
       <c r="K605" s="2" t="inlineStr">
         <is>
-          <t>Years of filings</t>
+          <t>Years of company filings. A limited company or LLP with 3+ years and active status gets category B.</t>
         </is>
       </c>
     </row>
@@ -28971,7 +29043,7 @@
       </c>
       <c r="K606" s="2" t="inlineStr">
         <is>
-          <t>Company status</t>
+          <t>ACTIVE | STRUCK_OFF | UNDER_INSOLVENCY | UNKNOWN. Struck-off or insolvent means category C and a person reviews.</t>
         </is>
       </c>
     </row>
@@ -29014,7 +29086,7 @@
       <c r="J607" s="2" t="inlineStr"/>
       <c r="K607" s="2" t="inlineStr">
         <is>
-          <t>Email domains</t>
+          <t>Official email domains, used to check the customer's work email.</t>
         </is>
       </c>
     </row>
@@ -29053,7 +29125,7 @@
       <c r="J608" s="2" t="inlineStr"/>
       <c r="K608" s="2" t="inlineStr">
         <is>
-          <t>Industry</t>
+          <t>Industry the employer works in.</t>
         </is>
       </c>
     </row>
@@ -29092,7 +29164,7 @@
       <c r="J609" s="2" t="inlineStr"/>
       <c r="K609" s="2" t="inlineStr">
         <is>
-          <t>Hq city</t>
+          <t>Head-office city.</t>
         </is>
       </c>
     </row>
@@ -29131,7 +29203,7 @@
       <c r="J610" s="2" t="inlineStr"/>
       <c r="K610" s="2" t="inlineStr">
         <is>
-          <t>Hq state</t>
+          <t>Head-office state, as a 2-letter code.</t>
         </is>
       </c>
     </row>
@@ -29174,7 +29246,7 @@
       <c r="J611" s="2" t="inlineStr"/>
       <c r="K611" s="2" t="inlineStr">
         <is>
-          <t>Caution</t>
+          <t>On the caution list; a case with this employer is referred to a person. Needs a reason.</t>
         </is>
       </c>
     </row>
@@ -29213,7 +29285,7 @@
       <c r="J612" s="2" t="inlineStr"/>
       <c r="K612" s="2" t="inlineStr">
         <is>
-          <t>Caution reason</t>
+          <t>Why the employer is on the caution list; required when caution is true.</t>
         </is>
       </c>
     </row>
@@ -29252,7 +29324,7 @@
       <c r="J613" s="2" t="inlineStr"/>
       <c r="K613" s="2" t="inlineStr">
         <is>
-          <t>When last verified</t>
+          <t>When the checks last ran on this employer.</t>
         </is>
       </c>
     </row>
@@ -29299,7 +29371,7 @@
       <c r="J614" s="2" t="inlineStr"/>
       <c r="K614" s="2" t="inlineStr">
         <is>
-          <t>Link to users.id</t>
+          <t>Staff user who last ran the checks; links to users.</t>
         </is>
       </c>
     </row>
@@ -29342,7 +29414,7 @@
       <c r="J615" s="2" t="inlineStr"/>
       <c r="K615" s="2" t="inlineStr">
         <is>
-          <t>Source</t>
+          <t>How the row was added: STAFF (added by staff) or FROM_APPLICATIONS (seeded from employer names on applications).</t>
         </is>
       </c>
     </row>
@@ -29385,7 +29457,7 @@
       <c r="J616" s="2" t="inlineStr"/>
       <c r="K616" s="2" t="inlineStr">
         <is>
-          <t>When the row was created</t>
+          <t>When the row was created.</t>
         </is>
       </c>
     </row>
@@ -29428,7 +29500,7 @@
       <c r="J617" s="2" t="inlineStr"/>
       <c r="K617" s="2" t="inlineStr">
         <is>
-          <t>When the row was last changed</t>
+          <t>When the row was last changed.</t>
         </is>
       </c>
     </row>
@@ -29475,7 +29547,7 @@
       <c r="J618" s="2" t="inlineStr"/>
       <c r="K618" s="2" t="inlineStr">
         <is>
-          <t>Internal key</t>
+          <t>Internal key.</t>
         </is>
       </c>
     </row>
@@ -29522,7 +29594,7 @@
       <c r="J619" s="2" t="inlineStr"/>
       <c r="K619" s="2" t="inlineStr">
         <is>
-          <t>Link to employers.id</t>
+          <t>Employer checked; links to employers. Rows are removed if the employer is deleted.</t>
         </is>
       </c>
     </row>
@@ -29565,7 +29637,7 @@
       </c>
       <c r="K620" s="2" t="inlineStr">
         <is>
-          <t>Check code</t>
+          <t>Which check: CIN_MCA | GSTIN | LISTED | GOVT_PSU | CAUTION.</t>
         </is>
       </c>
     </row>
@@ -29608,7 +29680,7 @@
       </c>
       <c r="K621" s="2" t="inlineStr">
         <is>
-          <t>Result</t>
+          <t>PASS | FAIL | REVIEW | NOT_APPLICABLE | INFO.</t>
         </is>
       </c>
     </row>
@@ -29651,7 +29723,7 @@
       <c r="J622" s="2" t="inlineStr"/>
       <c r="K622" s="2" t="inlineStr">
         <is>
-          <t>Detail</t>
+          <t>What the check compared and found (JSON).</t>
         </is>
       </c>
     </row>
@@ -29690,7 +29762,7 @@
       <c r="J623" s="2" t="inlineStr"/>
       <c r="K623" s="2" t="inlineStr">
         <is>
-          <t>Source</t>
+          <t>What answered the check, e.g. SIMULATED (company lookup), FORMAT, REFERENCE_LIST or MASTER.</t>
         </is>
       </c>
     </row>
@@ -29729,7 +29801,7 @@
       <c r="J624" s="2" t="inlineStr"/>
       <c r="K624" s="2" t="inlineStr">
         <is>
-          <t>Checked by</t>
+          <t>Staff user who ran the check.</t>
         </is>
       </c>
     </row>
@@ -29772,7 +29844,7 @@
       <c r="J625" s="2" t="inlineStr"/>
       <c r="K625" s="2" t="inlineStr">
         <is>
-          <t>When checked</t>
+          <t>When the check ran.</t>
         </is>
       </c>
     </row>
@@ -29819,7 +29891,7 @@
       <c r="J626" s="2" t="inlineStr"/>
       <c r="K626" s="2" t="inlineStr">
         <is>
-          <t>Internal key</t>
+          <t>Internal key.</t>
         </is>
       </c>
     </row>
@@ -29866,7 +29938,7 @@
       <c r="J627" s="2" t="inlineStr"/>
       <c r="K627" s="2" t="inlineStr">
         <is>
-          <t>Link to employers.id</t>
+          <t>Employer whose category would change; links to employers.</t>
         </is>
       </c>
     </row>
@@ -29905,7 +29977,7 @@
       <c r="J628" s="2" t="inlineStr"/>
       <c r="K628" s="2" t="inlineStr">
         <is>
-          <t>From category</t>
+          <t>Category at the time of the request.</t>
         </is>
       </c>
     </row>
@@ -29948,7 +30020,7 @@
       </c>
       <c r="K629" s="2" t="inlineStr">
         <is>
-          <t>To category</t>
+          <t>Category asked for: A | B | C.</t>
         </is>
       </c>
     </row>
@@ -29987,7 +30059,7 @@
       <c r="J630" s="2" t="inlineStr"/>
       <c r="K630" s="2" t="inlineStr">
         <is>
-          <t>Reason</t>
+          <t>Why the change is asked; requests raised by the checks quote the check outcome.</t>
         </is>
       </c>
     </row>
@@ -30034,7 +30106,7 @@
       </c>
       <c r="K631" s="2" t="inlineStr">
         <is>
-          <t>Status</t>
+          <t>PENDING | APPROVED | REJECTED | WITHDRAWN. Default PENDING; only one PENDING request per employer.</t>
         </is>
       </c>
     </row>
@@ -30073,7 +30145,7 @@
       <c r="J632" s="2" t="inlineStr"/>
       <c r="K632" s="2" t="inlineStr">
         <is>
-          <t>Requested by</t>
+          <t>Staff user who made the request.</t>
         </is>
       </c>
     </row>
@@ -30116,7 +30188,7 @@
       <c r="J633" s="2" t="inlineStr"/>
       <c r="K633" s="2" t="inlineStr">
         <is>
-          <t>When requested</t>
+          <t>When the request was made.</t>
         </is>
       </c>
     </row>
@@ -30155,7 +30227,7 @@
       <c r="J634" s="2" t="inlineStr"/>
       <c r="K634" s="2" t="inlineStr">
         <is>
-          <t>Decided by</t>
+          <t>Staff user who decided. Approve or reject must be a different person; only the requester can withdraw.</t>
         </is>
       </c>
     </row>
@@ -30194,7 +30266,7 @@
       <c r="J635" s="2" t="inlineStr"/>
       <c r="K635" s="2" t="inlineStr">
         <is>
-          <t>When decided</t>
+          <t>When the request was decided or withdrawn.</t>
         </is>
       </c>
     </row>
@@ -30233,7 +30305,7 @@
       <c r="J636" s="2" t="inlineStr"/>
       <c r="K636" s="2" t="inlineStr">
         <is>
-          <t>Decision note</t>
+          <t>Optional note from the person who decided.</t>
         </is>
       </c>
     </row>
@@ -30280,7 +30352,7 @@
       </c>
       <c r="K637" s="2" t="inlineStr">
         <is>
-          <t>List code</t>
+          <t>Which list: GOVT_PSU | LISTED. Part of the key.</t>
         </is>
       </c>
     </row>
@@ -30319,7 +30391,7 @@
       <c r="J638" s="2" t="inlineStr"/>
       <c r="K638" s="2" t="inlineStr">
         <is>
-          <t>Name</t>
+          <t>Name of the organisation on the list.</t>
         </is>
       </c>
     </row>
@@ -30362,7 +30434,7 @@
       <c r="J639" s="2" t="inlineStr"/>
       <c r="K639" s="2" t="inlineStr">
         <is>
-          <t>Name key</t>
+          <t>Normalised name (same rule as employers.name_key) used for matching. Part of the key.</t>
         </is>
       </c>
     </row>
@@ -30401,7 +30473,7 @@
       <c r="J640" s="2" t="inlineStr"/>
       <c r="K640" s="2" t="inlineStr">
         <is>
-          <t>Exchange</t>
+          <t>Stock exchange for a listed company, e.g. NSE or BSE.</t>
         </is>
       </c>
     </row>
@@ -30440,7 +30512,7 @@
       <c r="J641" s="2" t="inlineStr"/>
       <c r="K641" s="2" t="inlineStr">
         <is>
-          <t>Symbol</t>
+          <t>Stock symbol for a listed company.</t>
         </is>
       </c>
     </row>
@@ -30479,7 +30551,7 @@
       <c r="J642" s="2" t="inlineStr"/>
       <c r="K642" s="2" t="inlineStr">
         <is>
-          <t>Source</t>
+          <t>Where the entry came from, e.g. "Starting list, 3 Oct 2026".</t>
         </is>
       </c>
     </row>
@@ -30522,7 +30594,7 @@
       <c r="J643" s="2" t="inlineStr"/>
       <c r="K643" s="2" t="inlineStr">
         <is>
-          <t>When added</t>
+          <t>When the entry was added.</t>
         </is>
       </c>
     </row>
@@ -30569,7 +30641,7 @@
       <c r="J644" s="2" t="inlineStr"/>
       <c r="K644" s="2" t="inlineStr">
         <is>
-          <t>Internal key</t>
+          <t>Always true; the CHECK allows only one row.</t>
         </is>
       </c>
     </row>
@@ -30616,7 +30688,7 @@
       </c>
       <c r="K645" s="2" t="inlineStr">
         <is>
-          <t>Provider</t>
+          <t>SIMULATED | MCA_LIVE. SIMULATED reads the CIN's own fields and treats the company as active; it never invents facts.</t>
         </is>
       </c>
     </row>
@@ -30663,7 +30735,7 @@
       <c r="J646" s="2" t="inlineStr"/>
       <c r="K646" s="2" t="inlineStr">
         <is>
-          <t>Internal key</t>
+          <t>Internal key.</t>
         </is>
       </c>
     </row>
@@ -30706,7 +30778,7 @@
       </c>
       <c r="K647" s="2" t="inlineStr">
         <is>
-          <t>Category code</t>
+          <t>A | B | C. Unique together with policy_version.</t>
         </is>
       </c>
     </row>
@@ -30745,7 +30817,7 @@
       <c r="J648" s="2" t="inlineStr"/>
       <c r="K648" s="2" t="inlineStr">
         <is>
-          <t>Category label</t>
+          <t>Display name, e.g. Category A.</t>
         </is>
       </c>
     </row>
@@ -30784,7 +30856,7 @@
       <c r="J649" s="2" t="inlineStr"/>
       <c r="K649" s="2" t="inlineStr">
         <is>
-          <t>Description</t>
+          <t>Which employers fall in the category, e.g. listed companies, government, PSUs and large MNCs for A.</t>
         </is>
       </c>
     </row>
@@ -30827,7 +30899,7 @@
       <c r="J650" s="2" t="inlineStr"/>
       <c r="K650" s="2" t="inlineStr">
         <is>
-          <t>Rate loading pct</t>
+          <t>Added to the bureau band's base rate, in % points; 0 or more. Seed: A 0.00, B 0.40, C 1.25.</t>
         </is>
       </c>
     </row>
@@ -30866,7 +30938,7 @@
       <c r="J651" s="2" t="inlineStr"/>
       <c r="K651" s="2" t="inlineStr">
         <is>
-          <t>Max ltv pct</t>
+          <t>Highest loan-to-value allowed on the ex-showroom price, in %. Seed: A 120, B 110, C 90.</t>
         </is>
       </c>
     </row>
@@ -30905,7 +30977,7 @@
       <c r="J652" s="2" t="inlineStr"/>
       <c r="K652" s="2" t="inlineStr">
         <is>
-          <t>Max tenure months</t>
+          <t>Longest tenure allowed, in months. Seed: A 84, B 84, C 60.</t>
         </is>
       </c>
     </row>
@@ -30944,7 +31016,7 @@
       <c r="J653" s="2" t="inlineStr"/>
       <c r="K653" s="2" t="inlineStr">
         <is>
-          <t>Processing fee inr</t>
+          <t>Processing fee, in INR. Seed: A 5,000, B 6,500, C 8,000.</t>
         </is>
       </c>
     </row>
@@ -30983,7 +31055,7 @@
       <c r="J654" s="2" t="inlineStr"/>
       <c r="K654" s="2" t="inlineStr">
         <is>
-          <t>Display order</t>
+          <t>Order in which categories are shown on the rate grid page.</t>
         </is>
       </c>
     </row>
@@ -31022,7 +31094,7 @@
       <c r="J655" s="2" t="inlineStr"/>
       <c r="K655" s="2" t="inlineStr">
         <is>
-          <t>Policy version</t>
+          <t>Policy version these terms belong to, e.g. 2026.08.</t>
         </is>
       </c>
     </row>
@@ -31065,7 +31137,7 @@
       <c r="J656" s="2" t="inlineStr"/>
       <c r="K656" s="2" t="inlineStr">
         <is>
-          <t>Yes/no: active</t>
+          <t>Whether these terms are in use; default true.</t>
         </is>
       </c>
     </row>
@@ -31108,7 +31180,7 @@
       <c r="J657" s="2" t="inlineStr"/>
       <c r="K657" s="2" t="inlineStr">
         <is>
-          <t>When the row was created</t>
+          <t>When the row was created.</t>
         </is>
       </c>
     </row>
@@ -31151,7 +31223,7 @@
       <c r="J658" s="2" t="inlineStr"/>
       <c r="K658" s="2" t="inlineStr">
         <is>
-          <t>When the row was last changed</t>
+          <t>When the row was last changed; set automatically.</t>
         </is>
       </c>
     </row>

</xml_diff>